<commit_message>
Herken subtotalen in de config wizard en vink ze standaard uit
Een kolom is een subtotaal als de naam een woord als subtotaal/totaal/som
bevat, of als hij gelijk is aan de som van een aaneengesloten reeks andere
scorekolommen. De wizard vinkt die uit (met voorstellen ingevuld) en legt
in een tip uit dat een subtotaal naast zijn onderdelen dubbel telt.

De Leiden-democonfig neemt de twee subtotalen niet meer mee (9 items).

Deel van #38

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/demo/demo_leiden_2026/config.xlsx
+++ b/data/demo/demo_leiden_2026/config.xlsx
@@ -556,10 +556,6 @@
           <t>A_Nummer_Aanvraag</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="b">
@@ -570,10 +566,6 @@
           <t>Selectie</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="b">
@@ -584,10 +576,6 @@
           <t>A_Geslacht</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="b">
@@ -598,10 +586,6 @@
           <t>A_Gevolgde_Opleiding_1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="b">
@@ -627,7 +611,6 @@
           <t>Studieresultaat</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="b">
@@ -653,7 +636,6 @@
           <t>Studieresultaat</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="b">
@@ -664,10 +646,6 @@
           <t>A_Bachelor_Maanden_1</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="b">
@@ -678,10 +656,6 @@
           <t>A_Mnd_Nominaal1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="b">
@@ -692,10 +666,6 @@
           <t>A_Mnd_Ba_boven_Nominaal1</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="b">
@@ -706,10 +676,6 @@
           <t>A_Score_Duur_Ba_Nominaal1</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="b">
@@ -735,7 +701,6 @@
           <t>Studietempo</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="b">
@@ -746,10 +711,6 @@
           <t>B1_Achternaam</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="b">
@@ -760,10 +721,6 @@
           <t>B1_NL_Docs</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="b">
@@ -774,10 +731,6 @@
           <t>B1_Score_NL_Docs</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="b">
@@ -788,10 +741,6 @@
           <t>B1_NL_Gespr_Schrijf</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="b">
@@ -802,10 +751,6 @@
           <t>B1_Score_NL_Gespr_Schrijf</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="b">
@@ -816,10 +761,6 @@
           <t>B1_Beoord_Gespr_Schrijfop</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="b">
@@ -830,10 +771,6 @@
           <t>B1_Score_Beoord_Gesprek</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="b">
@@ -844,10 +781,6 @@
           <t>B2_Achternaam</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="b">
@@ -858,10 +791,6 @@
           <t>B2_NL_Docs</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="b">
@@ -872,10 +801,6 @@
           <t>B2_Score_NL_Docs</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="b">
@@ -886,10 +811,6 @@
           <t>B2_NL_Gespr_Schrijf</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="b">
@@ -900,10 +821,6 @@
           <t>B2_Score_NL_Gespr_Schrijf</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="b">
@@ -914,10 +831,6 @@
           <t>B2_Beoord_Gespr_Schrijfop</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="b">
@@ -928,10 +841,6 @@
           <t>B2_Score_Beoord_Gesprek</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="b">
@@ -942,10 +851,6 @@
           <t>C_Sc_Gem_Cijfer_Ba</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="b">
@@ -956,10 +861,6 @@
           <t>C_Sc_Duur_Ba_Nominaal1</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="b">
@@ -985,7 +886,6 @@
           <t>Taalbeheersing</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="b">
@@ -1011,7 +911,6 @@
           <t>Taalbeheersing</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="b">
@@ -1037,7 +936,6 @@
           <t>Taalbeheersing</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="b">
@@ -1063,7 +961,6 @@
           <t>Taalbeheersing</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="b">
@@ -1089,7 +986,6 @@
           <t>Communicatievaardigheid</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="b">
@@ -1115,7 +1011,6 @@
           <t>Communicatievaardigheid</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="b">
@@ -1126,10 +1021,6 @@
           <t>C_B1_Sc_SubTotaal</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="b">
@@ -1140,14 +1031,10 @@
           <t>C_B2_Sc_SubTotaal</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1164,12 +1051,10 @@
           <t>Subtotaal gesprek B1+B2</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1186,8 +1071,6 @@
           <t>Subtotaal diploma</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="b">
@@ -1198,10 +1081,6 @@
           <t>C_Sc_Totaal</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="b">
@@ -1212,10 +1091,6 @@
           <t>Rangnummer definitief</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>